<commit_message>
Viking Saç Tokası fiyat güncellemesi: 14K Altın → -, Gümüş Üzeri Altın Kaplama → 3.000 ₺
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aysegulkucukoglu/Documents/Rosary Claude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565B2AEB-91BB-6C4C-9B4F-4829B7BB6073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BBE44AD-5805-3049-A3FE-7EE97E9D0A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ürün Kataloğu" sheetId="1" r:id="rId1"/>
@@ -451,7 +451,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1917,11 +1924,11 @@
       <c r="H17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J17" s="5">
         <v>3000</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>84</v>
       </c>
       <c r="K17" s="7"/>
       <c r="L17" s="5"/>
@@ -1970,21 +1977,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{F33B7C9F-4EC9-3B46-B2F4-A55998A4C073}">
-            <xm:f>NOT(ISERROR(SEARCH("-",J1)))</xm:f>
-            <xm:f>"-"</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor theme="5" tint="0.59996337778862885"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>J2:K1048576 J1</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{A5B7E675-8585-AB41-A517-427893EDE478}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{A5B7E675-8585-AB41-A517-427893EDE478}">
             <xm:f>NOT(ISERROR(SEARCH("-",I13)))</xm:f>
             <xm:f>"-"</xm:f>
             <x14:dxf>
@@ -1997,6 +1990,34 @@
           </x14:cfRule>
           <xm:sqref>I13</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{F33B7C9F-4EC9-3B46-B2F4-A55998A4C073}">
+            <xm:f>NOT(ISERROR(SEARCH("-",J1)))</xm:f>
+            <xm:f>"-"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="5" tint="0.59996337778862885"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>J1 J2:K16 J18:K1048576 K17</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{8F1DD2CD-89CC-7C4B-A96A-36F05EEC4182}">
+            <xm:f>NOT(ISERROR(SEARCH("-",I17)))</xm:f>
+            <xm:f>"-"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="5" tint="0.59996337778862885"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>I17</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
Toi et Moi Renkli Taşlı Yüzük: açıklamaya sembolik anlam eklendi (aşk, bağlılık, eşit ortaklık)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -777,6 +777,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -802,6 +805,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2077,7 +2083,7 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>İki renkli değerli taşın yan yana yerleştirildiği bir Toi et Moi yüzük. 14K altın (sarı veya beyaz) ya da 925 gümüş üzeri 14K beyaz altın rodaj olarak üretilebilir.</t>
+          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki farklı taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte iki renkli değerli taş yan yana konumlanır. 14K altın (sarı veya beyaz) ya da 925 gümüş üzeri 14K beyaz altın rodaj olarak üretilebilir.</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Product #18 (Lab-Grown Toi et Moi): açıklamaya sembolik anlam eklendi + ana foto 5. foto yapıldı
- TR/EN desc: Toi et Moi sembolizmi (aşk, bağlılık, eşit ortaklık)
- Ana fotoğraf: nightjar_image_natural_light... → nightjar_image_image-j571jfggcgb65...
- Detay sayfası, koleksiyon kartı, ana sayfa featured-grid + Excel katalog güncellendi
- Yeni _sm versiyon oluşturuldu (mobil srcset için), eski silindi

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -760,13 +760,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -788,7 +788,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -805,9 +805,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2043,7 +2040,7 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Sertifikalı 1 ct ve 3 ct D/E renk lab-grown pırlantalarla üretilen bir Toi et Moi yüzük. Taşlar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak talep edilebilir.</t>
+          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte sertifikalı 1 ct ve 3 ct D/E renk lab-grown pırlantalar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak talep edilebilir.</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Product #19 (Colored Toi et Moi): ana foto 4. foto (colored4.jpeg) yapıldı
- Detay, kart, ana sayfa, meta og/twitter, Excel katalog güncellendi
- Yeni _sm versiyon oluşturuldu, eski silindi

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -760,7 +760,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -788,7 +788,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>

</xml_diff>

<commit_message>
Product #18 (Lab-Grown Toi et Moi): pırlantalar için 'IGI Sertifikalı' ibaresi eklendi
- translations.js (TR/EN): spec.stone + desc güncellendi
- HTML fallback metinleri (detay + koleksiyon + JSON-LD)
- Excel katalog: taş sütunu ve açıklama

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -805,6 +805,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2040,12 +2043,12 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte sertifikalı 1 ct ve 3 ct D/E renk lab-grown pırlantalar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak talep edilebilir.</t>
+          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte IGI sertifikalı 1 ct ve 3 ct D/E renk lab-grown pırlantalar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak talep edilebilir.</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Lab-Grown Pırlanta D/E, 1 ct + 3 ct (sertifikalı)</t>
+          <t>IGI Sertifikalı Lab-Grown Pırlanta D/E, 1 ct + 3 ct</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Product #18 (Lab-Grown Toi et Moi): main.png yeni ana foto — galeri, kart, ana sayfa, meta, Excel güncellendi
- main.png (28MB → 832KB) + main_sm.png (284KB) oluşturuldu
- Detay sayfası: ana görsel + thumbnails'in başına eklendi (aktif)
- Eski _sm dosyası (j571...) temizlendi

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -760,7 +760,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -788,7 +788,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -805,9 +805,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>

<commit_message>
Product #18: pırlanta karatı ve boyutları düzeltildi (0.9 ct 6.30 mm + 2.0 ct 12.00×7.00 mm)
- Önceki değer '1 ct + 3 ct' → gerçek IGI sertifika değerleri
- translations.js (TR + EN spec.stone ve desc)
- HTML fallback (detay + kart + JSON-LD + meta)
- Excel katalog (taş ve açıklama sütunları)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -805,6 +805,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2040,12 +2043,12 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte IGI sertifikalı 1 ct ve 3 ct D/E renk lab-grown pırlantalar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak sipariş verilebilir.</t>
+          <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte IGI sertifikalı 0.9 ct ve 2.0 ct D/E renk lab-grown pırlantalar 14K altın montür üzerinde birlikte oturtulmuştur. Sarı veya beyaz altın olarak sipariş verilebilir.</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>IGI Sertifikalı Lab-Grown Pırlanta D/E, 1 ct + 3 ct</t>
+          <t>IGI Sertifikalı Lab-Grown Pırlanta D/E, 0.9 ct (6.30 mm) + 2.0 ct (12.00 × 7.00 mm)</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Viking Saç Tokası güncellemesi:
- Fulltype: 'Zirkon Taşlı Altın Kaplama Saç Tokası' → 'Zirkon Taşlı Saç Tokası'
- 2 materyal seçeneği:
  - 925 Gümüş (Beyaz) — 2.000 ₺
  - Gümüş Üzeri Altın Kaplama (Sarı) — 3.000 ₺
- Yeni i18n key'ler: price.silverWhite, price.platedYellow (TR + EN)
- Pricing block detay + kart güncellendi
- Excel katalog: tür, materyal, fiyatlar güncel

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Zirkon Taşlı Altın Kaplama Saç Tokası</t>
+          <t>Zirkon Taşlı Saç Tokası</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1954,13 +1954,11 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>14K Altın / Kaplama</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>925 Gümüş / Gümüş Üzeri Altın Kaplama</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>2000</v>
       </c>
       <c r="J17" s="5" t="n">
         <v>3000</v>

</xml_diff>

<commit_message>
SEO: yeni ürün fotoğrafları SEO-uyumlu isimlere geçirildi
- Product 17: laser engrave pendant... → lazer-cizim-pirlantali-altin-kolye-ucu.jpeg
- Product 18 (Toi et Moi Lab-Grown): main.png → toi-et-moi-lab-grown-pirlanta-altin-yuzuk.png
  + 6 alt foto → toi-et-moi-lab-grown-pirlanta-yuzuk-{2..7}.jpeg
- Product 19 (Toi et Moi Coloured): colored4.jpeg → toi-et-moi-renkli-tasli-altin-yuzuk.jpeg
  + 2 alt foto → toi-et-moi-renkli-tasli-yuzuk-{2,3}.jpeg
- Toplam 15 dosya git mv ile yeniden adlandırıldı
- HTML/CSS/JS'te tüm referanslar güncellendi (raw + URL-encoded)
- Excel katalogda thumbnail'ler yeni dosyalardan üretildi
- Google image search'te ilgili keyword'lerde bulunabilirlik artacak

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -736,7 +736,7 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 17" descr="Picture"/>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -746,12 +746,32 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -770,34 +790,6 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>18</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
         <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
@@ -805,9 +797,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>

<commit_message>
SEO: 16 ürünün tüm resim dosyaları SEO-uyumlu isimlere geçirildi
- Ana foto: {slug}.{ext} (örn Product 12/gul-motifli-altin-kolye.jpg)
- Alt fotolar: {slug}-2, -3, ... alfabetik sırayla
- _sm mobil versiyonlar aynı slug ile eşleştirildi
- Toplam 82 dosya git mv ile yeniden adlandırıldı (tarih korundu)
- 27 HTML/CSS/JS dosyasında referanslar güncellendi (raw + URL-encoded)
- Excel katalog 16 ürün için yeni fotoğraflardan yenilendi
- Kök dizindeki story-beginning.webp bırakıldı (birden çok yerde kullanılıyor)

Google Image Search'te ürün, materyal ve motif anahtar kelimelerinde
görünürlük belirgin biçimde artacak.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -250,13 +250,13 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 1" descr="Picture"/>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -266,12 +266,91 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -286,22 +365,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 2" descr="Picture"/>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+        <a:blip cstate="print" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -316,22 +390,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Image 3" descr="Picture"/>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
+        <a:blip cstate="print" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -346,22 +415,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="5" name="Image 4" descr="Picture"/>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
+        <a:blip cstate="print" r:embed="rId7"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -376,22 +440,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 5" descr="Picture"/>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
+        <a:blip cstate="print" r:embed="rId8"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -406,22 +465,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 6" descr="Picture"/>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
+        <a:blip cstate="print" r:embed="rId9"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -436,22 +490,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 7" descr="Picture"/>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
+        <a:blip cstate="print" r:embed="rId10"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -466,22 +515,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Image 8" descr="Picture"/>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
+        <a:blip cstate="print" r:embed="rId11"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -496,22 +540,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 9" descr="Picture"/>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
+        <a:blip cstate="print" r:embed="rId12"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -526,22 +565,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="11" name="Image 10" descr="Picture"/>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
+        <a:blip cstate="print" r:embed="rId13"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -556,22 +590,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Image 11" descr="Picture"/>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
+        <a:blip cstate="print" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -586,22 +615,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Image 12" descr="Picture"/>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
+        <a:blip cstate="print" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -616,22 +640,17 @@
     <ext cx="1047750" cy="1047750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="14" name="Image 13" descr="Picture"/>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
+        <a:blip cstate="print" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,96 +660,6 @@
       <col>1</col>
       <colOff>0</colOff>
       <row>14</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>15</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>16</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -755,7 +684,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>
@@ -780,7 +709,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1047750" cy="1047750"/>

</xml_diff>

<commit_message>
Products 20-22 fiyat güncellemesi (Excel'e göre)
P20: 34.000 → 32.000, P21: 24.000 → 22.000, P22: 81.000/78.000 → 77.000/74.000. P23 ve P24 aynı kaldı. Detay HTML sayfaları, products.html kartları ve JSON-LD offers.price senkron.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aysegulkucukoglu/Documents/Rosary Claude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960AA6FC-08B9-6F40-93E1-91A95D7ABC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C3A545-BB5E-A843-B8D9-0DD377952410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -537,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -567,12 +567,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2422,167 +2416,155 @@
       </c>
     </row>
     <row r="21" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12">
+      <c r="A21" s="9">
         <v>20</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="I21" s="12">
-        <v>34000</v>
-      </c>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
+      <c r="I21" s="11">
+        <v>32000</v>
+      </c>
+      <c r="J21" s="11"/>
     </row>
     <row r="22" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="12">
+      <c r="A22" s="9">
         <v>21</v>
       </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="13" t="s">
+      <c r="B22" s="10"/>
+      <c r="C22" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="12">
-        <v>24000</v>
-      </c>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
+      <c r="I22" s="11">
+        <v>22000</v>
+      </c>
+      <c r="J22" s="11"/>
     </row>
     <row r="23" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12">
+      <c r="A23" s="9">
         <v>22</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13" t="s">
+      <c r="B23" s="10"/>
+      <c r="C23" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="H23" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="I23" s="12">
-        <v>81000</v>
-      </c>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12">
-        <v>78000</v>
-      </c>
-      <c r="L23" s="12"/>
-      <c r="M23" s="12" t="s">
+      <c r="I23" s="11">
+        <v>77000</v>
+      </c>
+      <c r="J23" s="11"/>
+      <c r="K23" s="4">
+        <v>74000</v>
+      </c>
+      <c r="M23" s="6" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="12">
+      <c r="A24" s="9">
         <v>23</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="13" t="s">
+      <c r="B24" s="10"/>
+      <c r="C24" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="F24" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="H24" s="13" t="s">
+      <c r="H24" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="11">
         <v>16000</v>
       </c>
-      <c r="J24" s="12">
+      <c r="J24" s="11">
         <v>18000</v>
       </c>
-      <c r="K24" s="12"/>
-      <c r="L24" s="12"/>
-      <c r="M24" s="12" t="s">
+      <c r="M24" s="6" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="12">
+      <c r="A25" s="9">
         <v>24</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13" t="s">
+      <c r="B25" s="10"/>
+      <c r="C25" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="F25" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="G25" s="13" t="s">
+      <c r="G25" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="H25" s="13" t="s">
+      <c r="H25" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="I25" s="12">
+      <c r="I25" s="11">
         <v>23000</v>
       </c>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="12"/>
+      <c r="J25" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Katalog güncellemeleri siteye yansıtıldı (fiyat + taş)
Ürün kataloğunda değişen alanlar senkronlandı:
- No 19 (Toi et Moi Renkli Taşlı Yüzük): 14K 46.000->24.000 ₺,
  Kaplama 14.000->9.000 ₺; taş "Renkli Doğal Taşlar (kuvars)".
- No 21 (Dalga Formlu Sade Yüzük): 14K 22.000->19.000 ₺.
- No 23 (Üçlü Renkli Doğal Taşlı Yüzük Seti): 925 Gümüş 16.000->9.000 ₺,
  Kaplama 18.000->11.000 ₺; taş "Renkli Doğal Taşlar (kuvars)".
Koleksiyon sayfası, ilgili ürün detay sayfaları ve TR/EN çeviriler güncellendi.
Güncel katalog dosyası da commit edildi (sonraki senkronlar için referans).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rosary-urun-katalogu.xlsx
+++ b/rosary-urun-katalogu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aysegulkucukoglu/Documents/Rosary Claude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C3A545-BB5E-A843-B8D9-0DD377952410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80ACAEFC-A253-8645-9AAB-43A67EEDC8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="135">
   <si>
     <t>No</t>
   </si>
@@ -360,9 +360,6 @@
     <t>Fransızca 'sen ve ben' anlamına gelen Toi et Moi, yan yana yerleştirilen iki farklı taşla iki ruhun bir araya gelişini anlatır; tarih boyunca aşkın, bağlılığın ve eşit ortaklığın simgesi olarak görülmüştür. Bu yüzükte iki renkli değerli taş yan yana konumlanır. 14K altın (sarı veya beyaz) ya da 925 gümüş üzeri 14K beyaz altın rodaj olarak üretilebilir.</t>
   </si>
   <si>
-    <t>Renkli Değerli Taşlar</t>
-  </si>
-  <si>
     <t>14K Altın (Sarı/Beyaz) / 925SS 14K Beyaz Altın Rodaj</t>
   </si>
   <si>
@@ -411,9 +408,6 @@
     <t>Dalga Formlu Üçlü Renkli Doğal Taşlı Yüzük Seti</t>
   </si>
   <si>
-    <t>Renkli Doğal Taşlar (ametist, kuvars, safir, yakut, zümrüt vb.)</t>
-  </si>
-  <si>
     <t>925 Gümüş / 925SS 14K Altın Kaplama (Sarı veya Beyaz)</t>
   </si>
   <si>
@@ -430,6 +424,9 @@
   </si>
   <si>
     <t>Üç dalga formlu yüzüğün, renkli doğal taşlarla süslendiği bir set. Birlikte ya da ayrı ayrı takılabilir; diğer dalga formlu modellerle kombin yapılabilir.</t>
+  </si>
+  <si>
+    <t>Renkli Doğal Taşlar (kuvars)</t>
   </si>
 </sst>
 </file>
@@ -537,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -566,6 +563,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1737,7 +1737,7 @@
     <col min="8" max="8" width="20" style="4" customWidth="1"/>
     <col min="9" max="9" width="18" style="4" customWidth="1"/>
     <col min="10" max="12" width="22" style="4" customWidth="1"/>
-    <col min="13" max="13" width="17.83203125" style="6" customWidth="1"/>
+    <col min="13" max="13" width="23.5" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="35" customHeight="1" x14ac:dyDescent="0.2">
@@ -2396,23 +2396,23 @@
       <c r="D20" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="12" t="s">
         <v>110</v>
       </c>
       <c r="F20" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="H20" s="11" t="s">
-        <v>113</v>
-      </c>
       <c r="I20" s="11">
-        <v>46000</v>
+        <v>24000</v>
       </c>
       <c r="J20" s="11">
-        <v>14000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
@@ -2421,22 +2421,22 @@
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="G21" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="H21" s="11" t="s">
         <v>117</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>118</v>
       </c>
       <c r="I21" s="11">
         <v>32000</v>
@@ -2449,25 +2449,25 @@
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>21</v>
       </c>
       <c r="E22" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="F22" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="G22" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="G22" s="11" t="s">
-        <v>122</v>
-      </c>
       <c r="H22" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I22" s="11">
-        <v>22000</v>
+        <v>19000</v>
       </c>
       <c r="J22" s="11"/>
     </row>
@@ -2477,22 +2477,22 @@
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="E23" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="F23" s="11" t="s">
         <v>125</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>126</v>
       </c>
       <c r="G23" s="11" t="s">
         <v>102</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I23" s="11">
         <v>77000</v>
@@ -2502,7 +2502,7 @@
         <v>74000</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
@@ -2511,31 +2511,31 @@
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D24" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="G24" s="11" t="s">
+      <c r="I24" s="11">
+        <v>9000</v>
+      </c>
+      <c r="J24" s="11">
+        <v>11000</v>
+      </c>
+      <c r="M24" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="H24" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="I24" s="11">
-        <v>16000</v>
-      </c>
-      <c r="J24" s="11">
-        <v>18000</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="95" customHeight="1" x14ac:dyDescent="0.2">
@@ -2544,22 +2544,22 @@
       </c>
       <c r="B25" s="10"/>
       <c r="C25" s="11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>21</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G25" s="11" t="s">
         <v>102</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I25" s="11">
         <v>23000</v>

</xml_diff>